<commit_message>
updated component list and powerpoint
</commit_message>
<xml_diff>
--- a/Fall 2025/Aero Design 1/Trade Studies/InterSat Link Trade Study.xlsx
+++ b/Fall 2025/Aero Design 1/Trade Studies/InterSat Link Trade Study.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noaht\School\Fall 2025\Aero Design 1\Trade Studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E5AA67F-2A1D-4D16-9158-53F7F5847ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10277A99-7328-4EEF-8529-10FDA08CB520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CBE0DF9F-DDFE-4833-8F35-1B1A204C32DC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="48">
   <si>
     <t>Part:</t>
   </si>
@@ -205,31 +205,34 @@
     <t>Communications</t>
   </si>
   <si>
-    <t>Power efficiency</t>
-  </si>
-  <si>
-    <t>Link Robustness</t>
-  </si>
-  <si>
-    <t>Antenna Size</t>
-  </si>
-  <si>
-    <t>Integration Effort</t>
-  </si>
-  <si>
-    <t>Sub-GHz GFSK (868/915 MHz)</t>
-  </si>
-  <si>
-    <t>2.4 GHz 802.15.4 / BLE</t>
-  </si>
-  <si>
-    <t>S-band low-power custom</t>
-  </si>
-  <si>
-    <t>UWB (Decawave)</t>
-  </si>
-  <si>
-    <t>Optical IR LED/PD</t>
+    <t>Robust/Herritage</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Short Range Sustainability</t>
+  </si>
+  <si>
+    <t>Integration</t>
+  </si>
+  <si>
+    <t>Mass/Vol</t>
+  </si>
+  <si>
+    <t>Tuning</t>
+  </si>
+  <si>
+    <t>ISIS Tape Spring</t>
+  </si>
+  <si>
+    <t>Oxford Deployable Helical</t>
+  </si>
+  <si>
+    <t>Antenna	Mech./Heritage (30)	Short-range Suitability (20)	Integration (20)	Mass/Vol (15)	Cost/Lead (10)	915 MHz Tuning (5)	Total /100
+ISIS Tape Spring	5 (150) – very proven, flown	2 (40) – optimized for 435 MHz, too long electrically for 915 unless redesigned	2 (40) – requires deploy, burn-wire, mechanical complexity	3 (45)	3 (30)	2 (10)	315
+NanoAvionics Turnstile	4 (120) – good heritage	3 (60) – designed for 435 MHz; splitter adds loss, overkill for 150 m	2 (40) – deploy + splitter integration	3 (45)	3 (30)	2 (10)	305
+AAC ANT-100 Static Whip</t>
   </si>
 </sst>
 </file>
@@ -687,7 +690,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -762,6 +765,30 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -792,56 +819,26 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1196,7 +1193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC4302AA-4CFD-4C9C-A5EA-EC60A679F4CF}">
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
@@ -1207,92 +1204,82 @@
     <col min="7" max="8" width="10.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="32"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C1" s="40"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="34"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C2" s="42"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="34"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C3" s="42"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="35">
+      <c r="B4" s="43">
         <v>45916</v>
       </c>
-      <c r="C4" s="36"/>
-    </row>
-    <row r="5" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
+      <c r="C4" s="44"/>
+    </row>
+    <row r="5" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="38"/>
+      <c r="B5" s="34"/>
       <c r="C5" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
       <c r="E8" s="11"/>
     </row>
-    <row r="9" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7"/>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="43"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="39" t="s">
-        <v>44</v>
-      </c>
-      <c r="J9" s="40"/>
-      <c r="K9" s="41"/>
-      <c r="L9" s="42" t="s">
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="M9" s="43"/>
-      <c r="N9" s="44"/>
-      <c r="O9" s="45" t="s">
+      <c r="G9" s="50"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="52" t="s">
+        <v>47</v>
+      </c>
+      <c r="J9" s="29"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="31" t="s">
         <v>46</v>
       </c>
-      <c r="P9" s="46"/>
-      <c r="Q9" s="47"/>
-      <c r="R9" s="42" t="s">
-        <v>47</v>
-      </c>
-      <c r="S9" s="43"/>
-      <c r="T9" s="44"/>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="M9" s="32"/>
+      <c r="N9" s="33"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
         <v>4</v>
       </c>
@@ -1332,32 +1319,14 @@
       <c r="N10" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="O10" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="P10" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q10" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="R10" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="S10" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="T10" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
         <v>39</v>
       </c>
       <c r="C11" s="22"/>
       <c r="D11" s="23">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>15</v>
@@ -1366,311 +1335,281 @@
         <v>5</v>
       </c>
       <c r="G11" s="24">
-        <f t="shared" ref="G11:G12" si="0">IF($E11="Y", F11/SUM($F11,$I11,$L11,$O11,$R11), (1/F11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.25</v>
+        <f>IF($E11="Y", F11/SUM($F11,$I11,$L11), (1/F11)/SUM(1/$F11,1/$I11,1/$L11))</f>
+        <v>0.41666666666666669</v>
       </c>
       <c r="H11" s="10">
         <f>G11*$D11</f>
-        <v>6.25</v>
+        <v>12.5</v>
       </c>
       <c r="I11" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J11" s="24">
-        <f t="shared" ref="J11:J12" si="1">IF($E11="Y", I11/SUM($F11,$I11,$L11,$O11,$R11), (1/I11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.2</v>
+        <f>IF($E11="Y", I11/SUM($F11,$I11,$L11), (1/I11)/SUM(1/$F11,1/$I11,1/$L11))</f>
+        <v>0.25</v>
       </c>
       <c r="K11" s="10">
         <f>J11*$D11</f>
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="L11" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M11" s="24">
-        <f t="shared" ref="M11:M12" si="2">IF($E11="Y", L11/SUM($F11,$I11,$L11,$O11,$R11), (1/L11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.15</v>
+        <f>IF($E11="Y", L11/SUM($F11,$I11,$L11), (1/L11)/SUM(1/$F11,1/$I11,1/$L11))</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="N11" s="10">
         <f>M11*$D11</f>
-        <v>3.75</v>
-      </c>
-      <c r="O11" s="5">
-        <v>3</v>
-      </c>
-      <c r="P11" s="24">
-        <f t="shared" ref="P11:P12" si="3">IF($E11="Y", O11/SUM($F11,$I11,$L11,$O11,$R11), (1/O11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.15</v>
-      </c>
-      <c r="Q11" s="10">
-        <f>P11*$D11</f>
-        <v>3.75</v>
-      </c>
-      <c r="R11" s="5">
-        <v>5</v>
-      </c>
-      <c r="S11" s="24">
-        <f t="shared" ref="S11:S12" si="4">IF($E11="Y", R11/SUM($F11,$I11,$L11,$O11,$R11), (1/R11)/SUM(1/$F11,1/$I11,1/$L11,1/$O11,1/$R11))</f>
-        <v>0.25</v>
-      </c>
-      <c r="T11" s="10">
-        <f>S11*$D11</f>
-        <v>6.25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B12" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" s="24"/>
       <c r="D12" s="23">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="5">
+        <v>2</v>
+      </c>
+      <c r="G12" s="24">
+        <f t="shared" ref="G12:G16" si="0">IF($E12="Y", F12/SUM($F12,$I12,$L12), (1/F12)/SUM(1/$F12,1/$I12,1/$L12))</f>
+        <v>0.18181818181818182</v>
+      </c>
+      <c r="H12" s="10">
+        <f>G12*$D12</f>
+        <v>3.6363636363636367</v>
+      </c>
+      <c r="I12" s="5">
+        <v>4</v>
+      </c>
+      <c r="J12" s="24">
+        <f t="shared" ref="J12:J16" si="1">IF($E12="Y", I12/SUM($F12,$I12,$L12), (1/I12)/SUM(1/$F12,1/$I12,1/$L12))</f>
+        <v>0.36363636363636365</v>
+      </c>
+      <c r="K12" s="10">
+        <f>J12*$D12</f>
+        <v>7.2727272727272734</v>
+      </c>
+      <c r="L12" s="5">
         <v>5</v>
       </c>
-      <c r="G12" s="24">
+      <c r="M12" s="24">
+        <f t="shared" ref="M12:M16" si="2">IF($E12="Y", L12/SUM($F12,$I12,$L12), (1/L12)/SUM(1/$F12,1/$I12,1/$L12))</f>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="N12" s="10">
+        <f>M12*$D12</f>
+        <v>9.0909090909090899</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="24"/>
+      <c r="D13" s="23">
+        <v>20</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="5">
+        <v>2</v>
+      </c>
+      <c r="G13" s="24">
+        <f t="shared" si="0"/>
+        <v>0.2</v>
+      </c>
+      <c r="H13" s="10">
+        <f>G13*$D13</f>
+        <v>4</v>
+      </c>
+      <c r="I13" s="5">
+        <v>5</v>
+      </c>
+      <c r="J13" s="24">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="K13" s="10">
+        <f>J13*$D13</f>
+        <v>10</v>
+      </c>
+      <c r="L13" s="5">
+        <v>3</v>
+      </c>
+      <c r="M13" s="24">
+        <f t="shared" si="2"/>
+        <v>0.3</v>
+      </c>
+      <c r="N13" s="10">
+        <f>M13*$D13</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="24"/>
+      <c r="D14" s="23">
+        <v>15</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="5">
+        <v>3</v>
+      </c>
+      <c r="G14" s="24">
+        <f t="shared" si="0"/>
+        <v>0.27272727272727271</v>
+      </c>
+      <c r="H14" s="10"/>
+      <c r="I14" s="5">
+        <v>5</v>
+      </c>
+      <c r="J14" s="24">
+        <f t="shared" si="1"/>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="K14" s="10"/>
+      <c r="L14" s="5">
+        <v>3</v>
+      </c>
+      <c r="M14" s="24">
+        <f t="shared" si="2"/>
+        <v>0.27272727272727271</v>
+      </c>
+      <c r="N14" s="10"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="24"/>
+      <c r="D15" s="23">
+        <v>10</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="5">
+        <v>3</v>
+      </c>
+      <c r="G15" s="24">
         <f t="shared" si="0"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="H12" s="10">
-        <f>G12*$D12</f>
-        <v>8.3333333333333321</v>
-      </c>
-      <c r="I12" s="5">
-        <v>3</v>
-      </c>
-      <c r="J12" s="24">
+      <c r="H15" s="10"/>
+      <c r="I15" s="5">
+        <v>4</v>
+      </c>
+      <c r="J15" s="24">
         <f t="shared" si="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="K12" s="10">
-        <f>J12*$D12</f>
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="K15" s="10"/>
+      <c r="L15" s="5">
+        <v>2</v>
+      </c>
+      <c r="M15" s="24">
+        <f t="shared" si="2"/>
+        <v>0.22222222222222221</v>
+      </c>
+      <c r="N15" s="10"/>
+    </row>
+    <row r="16" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="24"/>
+      <c r="D16" s="23">
         <v>5</v>
       </c>
-      <c r="L12" s="5">
-        <v>3</v>
-      </c>
-      <c r="M12" s="24">
+      <c r="E16" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="5">
+        <v>2</v>
+      </c>
+      <c r="G16" s="24">
+        <f t="shared" si="0"/>
+        <v>0.18181818181818182</v>
+      </c>
+      <c r="H16" s="10">
+        <f>G16*$D16</f>
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="I16" s="5">
+        <v>4</v>
+      </c>
+      <c r="J16" s="24">
+        <f t="shared" si="1"/>
+        <v>0.36363636363636365</v>
+      </c>
+      <c r="K16" s="10">
+        <f>J16*$D16</f>
+        <v>1.8181818181818183</v>
+      </c>
+      <c r="L16" s="5">
+        <v>5</v>
+      </c>
+      <c r="M16" s="24">
         <f t="shared" si="2"/>
-        <v>0.2</v>
-      </c>
-      <c r="N12" s="10">
-        <f>M12*$D12</f>
-        <v>5</v>
-      </c>
-      <c r="O12" s="5">
-        <v>3</v>
-      </c>
-      <c r="P12" s="24">
-        <f t="shared" si="3"/>
-        <v>0.2</v>
-      </c>
-      <c r="Q12" s="10">
-        <f>P12*$D12</f>
-        <v>5</v>
-      </c>
-      <c r="R12" s="5">
-        <v>1</v>
-      </c>
-      <c r="S12" s="24">
-        <f t="shared" si="4"/>
-        <v>6.6666666666666666E-2</v>
-      </c>
-      <c r="T12" s="10">
-        <f>S12*$D12</f>
-        <v>1.6666666666666667</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="B13" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="23">
-        <v>10</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="5">
-        <v>4</v>
-      </c>
-      <c r="G13" s="24">
-        <f t="shared" ref="G13:G14" si="5">IF($E13="Y", F13/SUM($F13,$I13,$L13,$O13,$R13), (1/F13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.2</v>
-      </c>
-      <c r="H13" s="10">
-        <f>G13*$D13</f>
-        <v>2</v>
-      </c>
-      <c r="I13" s="5">
-        <v>5</v>
-      </c>
-      <c r="J13" s="24">
-        <f t="shared" ref="J13:J14" si="6">IF($E13="Y", I13/SUM($F13,$I13,$L13,$O13,$R13), (1/I13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.25</v>
-      </c>
-      <c r="K13" s="10">
-        <f>J13*$D13</f>
-        <v>2.5</v>
-      </c>
-      <c r="L13" s="5">
-        <v>3</v>
-      </c>
-      <c r="M13" s="24">
-        <f t="shared" ref="M13:M14" si="7">IF($E13="Y", L13/SUM($F13,$I13,$L13,$O13,$R13), (1/L13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.15</v>
-      </c>
-      <c r="N13" s="10">
-        <f>M13*$D13</f>
-        <v>1.5</v>
-      </c>
-      <c r="O13" s="5">
-        <v>4</v>
-      </c>
-      <c r="P13" s="24">
-        <f t="shared" ref="P13:P14" si="8">IF($E13="Y", O13/SUM($F13,$I13,$L13,$O13,$R13), (1/O13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.2</v>
-      </c>
-      <c r="Q13" s="10">
-        <f>P13*$D13</f>
-        <v>2</v>
-      </c>
-      <c r="R13" s="5">
-        <v>4</v>
-      </c>
-      <c r="S13" s="24">
-        <f t="shared" ref="S13:S14" si="9">IF($E13="Y", R13/SUM($F13,$I13,$L13,$O13,$R13), (1/R13)/SUM(1/$F13,1/$I13,1/$L13,1/$O13,1/$R13))</f>
-        <v>0.2</v>
-      </c>
-      <c r="T13" s="10">
-        <f>S13*$D13</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="24"/>
-      <c r="D14" s="23">
-        <v>10</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="5">
-        <v>4</v>
-      </c>
-      <c r="G14" s="24">
-        <f t="shared" si="5"/>
-        <v>0.26666666666666666</v>
-      </c>
-      <c r="H14" s="10">
-        <f>G14*$D14</f>
-        <v>2.6666666666666665</v>
-      </c>
-      <c r="I14" s="5">
-        <v>4</v>
-      </c>
-      <c r="J14" s="24">
-        <f t="shared" si="6"/>
-        <v>0.26666666666666666</v>
-      </c>
-      <c r="K14" s="10">
-        <f>J14*$D14</f>
-        <v>2.6666666666666665</v>
-      </c>
-      <c r="L14" s="5">
-        <v>2</v>
-      </c>
-      <c r="M14" s="24">
-        <f t="shared" si="7"/>
-        <v>0.13333333333333333</v>
-      </c>
-      <c r="N14" s="10">
-        <f>M14*$D14</f>
-        <v>1.3333333333333333</v>
-      </c>
-      <c r="O14" s="5">
-        <v>2</v>
-      </c>
-      <c r="P14" s="24">
-        <f t="shared" si="8"/>
-        <v>0.13333333333333333</v>
-      </c>
-      <c r="Q14" s="10">
-        <f>P14*$D14</f>
-        <v>1.3333333333333333</v>
-      </c>
-      <c r="R14" s="5">
-        <v>3</v>
-      </c>
-      <c r="S14" s="24">
-        <f t="shared" si="9"/>
-        <v>0.2</v>
-      </c>
-      <c r="T14" s="10">
-        <f>S14*$D14</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="28" t="s">
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="N16" s="10">
+        <f>M16*$D16</f>
+        <v>2.2727272727272725</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="27">
-        <f>SUM(H11:H14)</f>
-        <v>19.25</v>
-      </c>
-      <c r="I15" s="13"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="27">
-        <f>SUM(K11:K14)</f>
-        <v>15.166666666666666</v>
-      </c>
-      <c r="L15" s="13"/>
-      <c r="M15" s="14"/>
-      <c r="N15" s="27">
-        <f>SUM(N11:N14)</f>
-        <v>11.583333333333334</v>
-      </c>
-      <c r="O15" s="13"/>
-      <c r="P15" s="14"/>
-      <c r="Q15" s="27">
-        <f>SUM(Q11:Q14)</f>
-        <v>12.083333333333334</v>
-      </c>
-      <c r="R15" s="13"/>
-      <c r="S15" s="14"/>
-      <c r="T15" s="27">
-        <f>SUM(T11:T14)</f>
-        <v>11.916666666666668</v>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="27">
+        <f>SUM(H11:H16)</f>
+        <v>21.045454545454547</v>
+      </c>
+      <c r="I17" s="13"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="27">
+        <f>SUM(K11:K16)</f>
+        <v>26.590909090909093</v>
+      </c>
+      <c r="L17" s="13"/>
+      <c r="M17" s="14"/>
+      <c r="N17" s="27">
+        <f>SUM(N11:N16)</f>
+        <v>27.363636363636363</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="L9:N9"/>
-    <mergeCell ref="O9:Q9"/>
-    <mergeCell ref="R9:T9"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="B15:E15"/>
+  <mergeCells count="10">
+    <mergeCell ref="B17:E17"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="F9:H9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1767,22 +1706,22 @@
     </row>
     <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="49" t="s">
+      <c r="B16" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="50"/>
-      <c r="D16" s="50"/>
-      <c r="E16" s="51"/>
-      <c r="F16" s="52" t="s">
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="53"/>
-      <c r="H16" s="54"/>
-      <c r="I16" s="39" t="s">
+      <c r="G16" s="50"/>
+      <c r="H16" s="51"/>
+      <c r="I16" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="J16" s="40"/>
-      <c r="K16" s="41"/>
+      <c r="J16" s="29"/>
+      <c r="K16" s="30"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
@@ -1889,12 +1828,12 @@
       </c>
     </row>
     <row r="20" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="30"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="38"/>
       <c r="F20" s="13"/>
       <c r="G20" s="14"/>
       <c r="H20" s="27">
@@ -1925,26 +1864,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="37bd234a-b872-4d8f-a05f-9ce9a06b0a24" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="619bfd31-fbc9-4e3d-b639-5680fd0427c3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100445E206EC97B5241AE364FC742D190F1" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8284591227d7a4ff90c48262bf6356f1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="619bfd31-fbc9-4e3d-b639-5680fd0427c3" xmlns:ns3="37bd234a-b872-4d8f-a05f-9ce9a06b0a24" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b29a3fb53242aaf6387bf4e700398a19" ns2:_="" ns3:_="">
     <xsd:import namespace="619bfd31-fbc9-4e3d-b639-5680fd0427c3"/>
@@ -2199,10 +2118,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="37bd234a-b872-4d8f-a05f-9ce9a06b0a24" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="619bfd31-fbc9-4e3d-b639-5680fd0427c3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1748E98C-71FF-4E5A-BAD7-3F9220D62AE3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F6E05F-13AA-425A-905B-6BF8E82F9AC9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="619bfd31-fbc9-4e3d-b639-5680fd0427c3"/>
+    <ds:schemaRef ds:uri="37bd234a-b872-4d8f-a05f-9ce9a06b0a24"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2225,20 +2175,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F6E05F-13AA-425A-905B-6BF8E82F9AC9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1748E98C-71FF-4E5A-BAD7-3F9220D62AE3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="619bfd31-fbc9-4e3d-b639-5680fd0427c3"/>
-    <ds:schemaRef ds:uri="37bd234a-b872-4d8f-a05f-9ce9a06b0a24"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>